<commit_message>
BASE COM OS DADOS ACRESCENTADOS - AC3
</commit_message>
<xml_diff>
--- a/Base_Vendas.xlsx
+++ b/Base_Vendas.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eugio\OneDrive\Documentos\Projeto TCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F8D950-22CF-4382-9249-9A9B28769417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77695C9-0501-4B5F-99D3-4A2A6268F57F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{F77771E8-BDAA-4D8A-8293-B9330D7E319F}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Metas" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$E$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$G$174</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="20">
   <si>
     <t>Data</t>
   </si>
@@ -91,6 +92,15 @@
   <si>
     <t>Paraná</t>
   </si>
+  <si>
+    <t>Desconto</t>
+  </si>
+  <si>
+    <t>Comissão Vendedor</t>
+  </si>
+  <si>
+    <t>Meta</t>
+  </si>
 </sst>
 </file>
 
@@ -113,7 +123,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -123,6 +133,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -139,10 +155,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -478,10 +495,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8619DC5A-B133-4640-889F-547BAA264472}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:G174"/>
   <sheetFormatPr defaultColWidth="36.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -497,8 +514,14 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>45658</v>
       </c>
@@ -514,8 +537,14 @@
       <c r="E2">
         <v>120</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>45659</v>
       </c>
@@ -531,8 +560,14 @@
       <c r="E3">
         <v>300</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <v>8</v>
+      </c>
+      <c r="G3">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>45660</v>
       </c>
@@ -548,8 +583,14 @@
       <c r="E4">
         <v>80</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>45661</v>
       </c>
@@ -565,8 +606,14 @@
       <c r="E5">
         <v>250</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>45662</v>
       </c>
@@ -582,8 +629,14 @@
       <c r="E6">
         <v>150</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="G6">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>45663</v>
       </c>
@@ -599,8 +652,14 @@
       <c r="E7">
         <v>320</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>45664</v>
       </c>
@@ -616,8 +675,14 @@
       <c r="E8">
         <v>90</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>45665</v>
       </c>
@@ -633,8 +698,14 @@
       <c r="E9">
         <v>270</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="G9">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>45666</v>
       </c>
@@ -650,8 +721,14 @@
       <c r="E10">
         <v>110</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F10">
+        <v>10</v>
+      </c>
+      <c r="G10">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>45667</v>
       </c>
@@ -667,8 +744,14 @@
       <c r="E11">
         <v>340</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <v>8</v>
+      </c>
+      <c r="G11">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>45668</v>
       </c>
@@ -684,8 +767,14 @@
       <c r="E12">
         <v>70</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>45669</v>
       </c>
@@ -701,8 +790,14 @@
       <c r="E13">
         <v>260</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>45670</v>
       </c>
@@ -718,8 +813,14 @@
       <c r="E14">
         <v>130</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F14">
+        <v>10</v>
+      </c>
+      <c r="G14">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>45671</v>
       </c>
@@ -735,8 +836,14 @@
       <c r="E15">
         <v>310</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F15">
+        <v>8</v>
+      </c>
+      <c r="G15">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>45672</v>
       </c>
@@ -752,8 +859,14 @@
       <c r="E16">
         <v>85</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>45673</v>
       </c>
@@ -769,8 +882,14 @@
       <c r="E17">
         <v>290</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17">
+        <v>4</v>
+      </c>
+      <c r="G17">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>45674</v>
       </c>
@@ -786,8 +905,14 @@
       <c r="E18">
         <v>305</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <v>4</v>
+      </c>
+      <c r="G18">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>45675</v>
       </c>
@@ -803,8 +928,14 @@
       <c r="E19">
         <v>254</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F19">
+        <v>8</v>
+      </c>
+      <c r="G19">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>45676</v>
       </c>
@@ -820,8 +951,14 @@
       <c r="E20">
         <v>424</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20">
+        <v>10</v>
+      </c>
+      <c r="G20">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>45677</v>
       </c>
@@ -837,8 +974,14 @@
       <c r="E21">
         <v>88</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F21">
+        <v>4</v>
+      </c>
+      <c r="G21">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>45678</v>
       </c>
@@ -854,8 +997,14 @@
       <c r="E22">
         <v>410</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F22">
+        <v>10</v>
+      </c>
+      <c r="G22">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>45679</v>
       </c>
@@ -871,8 +1020,14 @@
       <c r="E23">
         <v>237</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>45680</v>
       </c>
@@ -888,8 +1043,14 @@
       <c r="E24">
         <v>187</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F24">
+        <v>10</v>
+      </c>
+      <c r="G24">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>45681</v>
       </c>
@@ -905,8 +1066,14 @@
       <c r="E25">
         <v>233</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>45682</v>
       </c>
@@ -922,8 +1089,14 @@
       <c r="E26">
         <v>242</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F26">
+        <v>10</v>
+      </c>
+      <c r="G26">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>45683</v>
       </c>
@@ -939,8 +1112,14 @@
       <c r="E27">
         <v>114</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27">
+        <v>8</v>
+      </c>
+      <c r="G27">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>45684</v>
       </c>
@@ -956,8 +1135,14 @@
       <c r="E28">
         <v>101</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F28">
+        <v>4</v>
+      </c>
+      <c r="G28">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>45685</v>
       </c>
@@ -973,8 +1158,14 @@
       <c r="E29">
         <v>343</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29">
+        <v>8</v>
+      </c>
+      <c r="G29">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>45686</v>
       </c>
@@ -990,8 +1181,14 @@
       <c r="E30">
         <v>356</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F30">
+        <v>4</v>
+      </c>
+      <c r="G30">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>45687</v>
       </c>
@@ -1007,8 +1204,14 @@
       <c r="E31">
         <v>120</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F31">
+        <v>8</v>
+      </c>
+      <c r="G31">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>45688</v>
       </c>
@@ -1024,8 +1227,14 @@
       <c r="E32">
         <v>307</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F32">
+        <v>8</v>
+      </c>
+      <c r="G32">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>45689</v>
       </c>
@@ -1041,8 +1250,14 @@
       <c r="E33">
         <v>301</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>45690</v>
       </c>
@@ -1058,8 +1273,14 @@
       <c r="E34">
         <v>472</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>45691</v>
       </c>
@@ -1075,8 +1296,14 @@
       <c r="E35">
         <v>208</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F35">
+        <v>4</v>
+      </c>
+      <c r="G35">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>45692</v>
       </c>
@@ -1092,8 +1319,14 @@
       <c r="E36">
         <v>264</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F36">
+        <v>8</v>
+      </c>
+      <c r="G36">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>45693</v>
       </c>
@@ -1109,8 +1342,14 @@
       <c r="E37">
         <v>296</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37">
+        <v>10</v>
+      </c>
+      <c r="G37">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>45694</v>
       </c>
@@ -1126,8 +1365,14 @@
       <c r="E38">
         <v>76</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F38">
+        <v>4</v>
+      </c>
+      <c r="G38">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>45695</v>
       </c>
@@ -1143,8 +1388,14 @@
       <c r="E39">
         <v>66</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F39">
+        <v>8</v>
+      </c>
+      <c r="G39">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>45696</v>
       </c>
@@ -1160,8 +1411,14 @@
       <c r="E40">
         <v>477</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>45697</v>
       </c>
@@ -1177,8 +1434,14 @@
       <c r="E41">
         <v>261</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F41">
+        <v>4</v>
+      </c>
+      <c r="G41">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>45698</v>
       </c>
@@ -1194,8 +1457,14 @@
       <c r="E42">
         <v>195</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F42">
+        <v>10</v>
+      </c>
+      <c r="G42">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>45699</v>
       </c>
@@ -1211,8 +1480,14 @@
       <c r="E43">
         <v>437</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F43">
+        <v>8</v>
+      </c>
+      <c r="G43">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>45700</v>
       </c>
@@ -1228,8 +1503,14 @@
       <c r="E44">
         <v>405</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>45701</v>
       </c>
@@ -1245,8 +1526,14 @@
       <c r="E45">
         <v>346</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F45">
+        <v>8</v>
+      </c>
+      <c r="G45">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45702</v>
       </c>
@@ -1262,8 +1549,14 @@
       <c r="E46">
         <v>250</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>45703</v>
       </c>
@@ -1279,8 +1572,14 @@
       <c r="E47">
         <v>142</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>45704</v>
       </c>
@@ -1296,8 +1595,14 @@
       <c r="E48">
         <v>205</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F48">
+        <v>4</v>
+      </c>
+      <c r="G48">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>45705</v>
       </c>
@@ -1313,8 +1618,14 @@
       <c r="E49">
         <v>292</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F49">
+        <v>8</v>
+      </c>
+      <c r="G49">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>45706</v>
       </c>
@@ -1330,8 +1641,14 @@
       <c r="E50">
         <v>299</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50">
+        <v>10</v>
+      </c>
+      <c r="G50">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>45707</v>
       </c>
@@ -1347,8 +1664,14 @@
       <c r="E51">
         <v>306</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51">
+        <v>4</v>
+      </c>
+      <c r="G51">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>45708</v>
       </c>
@@ -1364,8 +1687,14 @@
       <c r="E52">
         <v>192</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F52">
+        <v>4</v>
+      </c>
+      <c r="G52">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>45709</v>
       </c>
@@ -1381,8 +1710,14 @@
       <c r="E53">
         <v>482</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F53">
+        <v>10</v>
+      </c>
+      <c r="G53">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>45710</v>
       </c>
@@ -1398,8 +1733,14 @@
       <c r="E54">
         <v>123</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>45711</v>
       </c>
@@ -1415,8 +1756,14 @@
       <c r="E55">
         <v>218</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>45712</v>
       </c>
@@ -1432,8 +1779,14 @@
       <c r="E56">
         <v>154</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F56">
+        <v>8</v>
+      </c>
+      <c r="G56">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>45713</v>
       </c>
@@ -1449,8 +1802,14 @@
       <c r="E57">
         <v>427</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57">
+        <v>4</v>
+      </c>
+      <c r="G57">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>45714</v>
       </c>
@@ -1466,8 +1825,14 @@
       <c r="E58">
         <v>335</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F58">
+        <v>4</v>
+      </c>
+      <c r="G58">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>45715</v>
       </c>
@@ -1483,8 +1848,14 @@
       <c r="E59">
         <v>79</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F59">
+        <v>4</v>
+      </c>
+      <c r="G59">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>45716</v>
       </c>
@@ -1500,8 +1871,14 @@
       <c r="E60">
         <v>146</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F60">
+        <v>8</v>
+      </c>
+      <c r="G60">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>45717</v>
       </c>
@@ -1517,8 +1894,14 @@
       <c r="E61">
         <v>374</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61">
+        <v>10</v>
+      </c>
+      <c r="G61">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>45718</v>
       </c>
@@ -1534,8 +1917,14 @@
       <c r="E62">
         <v>71</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F62">
+        <v>4</v>
+      </c>
+      <c r="G62">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>45719</v>
       </c>
@@ -1551,8 +1940,14 @@
       <c r="E63">
         <v>262</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>45720</v>
       </c>
@@ -1568,8 +1963,14 @@
       <c r="E64">
         <v>218</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F64">
+        <v>8</v>
+      </c>
+      <c r="G64">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>45721</v>
       </c>
@@ -1585,8 +1986,14 @@
       <c r="E65">
         <v>402</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F65">
+        <v>8</v>
+      </c>
+      <c r="G65">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>45722</v>
       </c>
@@ -1602,8 +2009,14 @@
       <c r="E66">
         <v>233</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F66">
+        <v>8</v>
+      </c>
+      <c r="G66">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>45723</v>
       </c>
@@ -1619,8 +2032,14 @@
       <c r="E67">
         <v>173</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>45724</v>
       </c>
@@ -1636,8 +2055,14 @@
       <c r="E68">
         <v>383</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>45725</v>
       </c>
@@ -1653,8 +2078,14 @@
       <c r="E69">
         <v>471</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F69">
+        <v>4</v>
+      </c>
+      <c r="G69">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>45726</v>
       </c>
@@ -1670,8 +2101,14 @@
       <c r="E70">
         <v>176</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F70">
+        <v>8</v>
+      </c>
+      <c r="G70">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>45727</v>
       </c>
@@ -1687,8 +2124,14 @@
       <c r="E71">
         <v>325</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F71">
+        <v>10</v>
+      </c>
+      <c r="G71">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>45728</v>
       </c>
@@ -1704,8 +2147,14 @@
       <c r="E72">
         <v>362</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F72">
+        <v>10</v>
+      </c>
+      <c r="G72">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>45729</v>
       </c>
@@ -1721,8 +2170,14 @@
       <c r="E73">
         <v>413</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F73">
+        <v>0</v>
+      </c>
+      <c r="G73">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>45730</v>
       </c>
@@ -1738,8 +2193,14 @@
       <c r="E74">
         <v>411</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74">
+        <v>0</v>
+      </c>
+      <c r="G74">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>45731</v>
       </c>
@@ -1755,8 +2216,14 @@
       <c r="E75">
         <v>438</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F75">
+        <v>4</v>
+      </c>
+      <c r="G75">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>45732</v>
       </c>
@@ -1772,8 +2239,14 @@
       <c r="E76">
         <v>98</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F76">
+        <v>10</v>
+      </c>
+      <c r="G76">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>45733</v>
       </c>
@@ -1789,8 +2262,14 @@
       <c r="E77">
         <v>364</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F77">
+        <v>10</v>
+      </c>
+      <c r="G77">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>45734</v>
       </c>
@@ -1806,8 +2285,14 @@
       <c r="E78">
         <v>177</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F78">
+        <v>10</v>
+      </c>
+      <c r="G78">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>45735</v>
       </c>
@@ -1823,8 +2308,14 @@
       <c r="E79">
         <v>123</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F79">
+        <v>0</v>
+      </c>
+      <c r="G79">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>45736</v>
       </c>
@@ -1840,8 +2331,14 @@
       <c r="E80">
         <v>193</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F80">
+        <v>8</v>
+      </c>
+      <c r="G80">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>45737</v>
       </c>
@@ -1857,8 +2354,14 @@
       <c r="E81">
         <v>68</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F81">
+        <v>0</v>
+      </c>
+      <c r="G81">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>45738</v>
       </c>
@@ -1874,8 +2377,14 @@
       <c r="E82">
         <v>187</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F82">
+        <v>4</v>
+      </c>
+      <c r="G82">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>45739</v>
       </c>
@@ -1891,8 +2400,14 @@
       <c r="E83">
         <v>339</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F83">
+        <v>0</v>
+      </c>
+      <c r="G83">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>45740</v>
       </c>
@@ -1908,8 +2423,14 @@
       <c r="E84">
         <v>383</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F84">
+        <v>0</v>
+      </c>
+      <c r="G84">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>45741</v>
       </c>
@@ -1925,8 +2446,14 @@
       <c r="E85">
         <v>403</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F85">
+        <v>8</v>
+      </c>
+      <c r="G85">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>45742</v>
       </c>
@@ -1942,8 +2469,14 @@
       <c r="E86">
         <v>497</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F86">
+        <v>4</v>
+      </c>
+      <c r="G86">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>45743</v>
       </c>
@@ -1959,8 +2492,14 @@
       <c r="E87">
         <v>237</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F87">
+        <v>4</v>
+      </c>
+      <c r="G87">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>45744</v>
       </c>
@@ -1976,8 +2515,14 @@
       <c r="E88">
         <v>54</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F88">
+        <v>0</v>
+      </c>
+      <c r="G88">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>45745</v>
       </c>
@@ -1993,8 +2538,14 @@
       <c r="E89">
         <v>125</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F89">
+        <v>10</v>
+      </c>
+      <c r="G89">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>45746</v>
       </c>
@@ -2010,8 +2561,14 @@
       <c r="E90">
         <v>254</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F90">
+        <v>10</v>
+      </c>
+      <c r="G90">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>45747</v>
       </c>
@@ -2027,8 +2584,14 @@
       <c r="E91">
         <v>102</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F91">
+        <v>4</v>
+      </c>
+      <c r="G91">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>45748</v>
       </c>
@@ -2044,8 +2607,14 @@
       <c r="E92">
         <v>361</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F92">
+        <v>8</v>
+      </c>
+      <c r="G92">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>45749</v>
       </c>
@@ -2061,8 +2630,14 @@
       <c r="E93">
         <v>104</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F93">
+        <v>10</v>
+      </c>
+      <c r="G93">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>45750</v>
       </c>
@@ -2078,8 +2653,14 @@
       <c r="E94">
         <v>243</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F94">
+        <v>0</v>
+      </c>
+      <c r="G94">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>45751</v>
       </c>
@@ -2095,8 +2676,14 @@
       <c r="E95">
         <v>51</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F95">
+        <v>8</v>
+      </c>
+      <c r="G95">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>45752</v>
       </c>
@@ -2112,8 +2699,14 @@
       <c r="E96">
         <v>265</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F96">
+        <v>10</v>
+      </c>
+      <c r="G96">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>45753</v>
       </c>
@@ -2129,8 +2722,14 @@
       <c r="E97">
         <v>364</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F97">
+        <v>10</v>
+      </c>
+      <c r="G97">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>45754</v>
       </c>
@@ -2146,8 +2745,14 @@
       <c r="E98">
         <v>427</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F98">
+        <v>0</v>
+      </c>
+      <c r="G98">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>45755</v>
       </c>
@@ -2163,8 +2768,14 @@
       <c r="E99">
         <v>480</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F99">
+        <v>4</v>
+      </c>
+      <c r="G99">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>45756</v>
       </c>
@@ -2180,8 +2791,14 @@
       <c r="E100">
         <v>108</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F100">
+        <v>10</v>
+      </c>
+      <c r="G100">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>45757</v>
       </c>
@@ -2197,16 +2814,1755 @@
       <c r="E101">
         <v>385</v>
       </c>
+      <c r="F101">
+        <v>8</v>
+      </c>
+      <c r="G101">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>46113</v>
+      </c>
+      <c r="B102" t="s">
+        <v>11</v>
+      </c>
+      <c r="C102" t="s">
+        <v>16</v>
+      </c>
+      <c r="D102" t="s">
+        <v>12</v>
+      </c>
+      <c r="E102">
+        <v>250</v>
+      </c>
+      <c r="F102">
+        <v>4</v>
+      </c>
+      <c r="G102">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B103" t="s">
+        <v>11</v>
+      </c>
+      <c r="C103" t="s">
+        <v>16</v>
+      </c>
+      <c r="D103" t="s">
+        <v>12</v>
+      </c>
+      <c r="E103">
+        <v>270</v>
+      </c>
+      <c r="F103">
+        <v>4</v>
+      </c>
+      <c r="G103">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>46115</v>
+      </c>
+      <c r="B104" t="s">
+        <v>11</v>
+      </c>
+      <c r="C104" t="s">
+        <v>16</v>
+      </c>
+      <c r="D104" t="s">
+        <v>12</v>
+      </c>
+      <c r="E104">
+        <v>260</v>
+      </c>
+      <c r="F104">
+        <v>4</v>
+      </c>
+      <c r="G104">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>46116</v>
+      </c>
+      <c r="B105" t="s">
+        <v>11</v>
+      </c>
+      <c r="C105" t="s">
+        <v>16</v>
+      </c>
+      <c r="D105" t="s">
+        <v>12</v>
+      </c>
+      <c r="E105">
+        <v>290</v>
+      </c>
+      <c r="F105">
+        <v>4</v>
+      </c>
+      <c r="G105">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>46117</v>
+      </c>
+      <c r="B106" t="s">
+        <v>7</v>
+      </c>
+      <c r="C106" t="s">
+        <v>16</v>
+      </c>
+      <c r="D106" t="s">
+        <v>6</v>
+      </c>
+      <c r="E106">
+        <v>305</v>
+      </c>
+      <c r="F106">
+        <v>4</v>
+      </c>
+      <c r="G106">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B107" t="s">
+        <v>5</v>
+      </c>
+      <c r="C107" t="s">
+        <v>16</v>
+      </c>
+      <c r="D107" t="s">
+        <v>8</v>
+      </c>
+      <c r="E107">
+        <v>88</v>
+      </c>
+      <c r="F107">
+        <v>4</v>
+      </c>
+      <c r="G107">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>46119</v>
+      </c>
+      <c r="B108" t="s">
+        <v>5</v>
+      </c>
+      <c r="C108" t="s">
+        <v>16</v>
+      </c>
+      <c r="D108" t="s">
+        <v>8</v>
+      </c>
+      <c r="E108">
+        <v>101</v>
+      </c>
+      <c r="F108">
+        <v>4</v>
+      </c>
+      <c r="G108">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>46120</v>
+      </c>
+      <c r="B109" t="s">
+        <v>5</v>
+      </c>
+      <c r="C109" t="s">
+        <v>16</v>
+      </c>
+      <c r="D109" t="s">
+        <v>10</v>
+      </c>
+      <c r="E109">
+        <v>356</v>
+      </c>
+      <c r="F109">
+        <v>4</v>
+      </c>
+      <c r="G109">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B110" t="s">
+        <v>9</v>
+      </c>
+      <c r="C110" t="s">
+        <v>16</v>
+      </c>
+      <c r="D110" t="s">
+        <v>8</v>
+      </c>
+      <c r="E110">
+        <v>208</v>
+      </c>
+      <c r="F110">
+        <v>4</v>
+      </c>
+      <c r="G110">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>46122</v>
+      </c>
+      <c r="B111" t="s">
+        <v>7</v>
+      </c>
+      <c r="C111" t="s">
+        <v>16</v>
+      </c>
+      <c r="D111" t="s">
+        <v>6</v>
+      </c>
+      <c r="E111">
+        <v>76</v>
+      </c>
+      <c r="F111">
+        <v>4</v>
+      </c>
+      <c r="G111">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>46123</v>
+      </c>
+      <c r="B112" t="s">
+        <v>7</v>
+      </c>
+      <c r="C112" t="s">
+        <v>16</v>
+      </c>
+      <c r="D112" t="s">
+        <v>6</v>
+      </c>
+      <c r="E112">
+        <v>261</v>
+      </c>
+      <c r="F112">
+        <v>4</v>
+      </c>
+      <c r="G112">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>46124</v>
+      </c>
+      <c r="B113" t="s">
+        <v>7</v>
+      </c>
+      <c r="C113" t="s">
+        <v>16</v>
+      </c>
+      <c r="D113" t="s">
+        <v>6</v>
+      </c>
+      <c r="E113">
+        <v>205</v>
+      </c>
+      <c r="F113">
+        <v>4</v>
+      </c>
+      <c r="G113">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>46125</v>
+      </c>
+      <c r="B114" t="s">
+        <v>11</v>
+      </c>
+      <c r="C114" t="s">
+        <v>16</v>
+      </c>
+      <c r="D114" t="s">
+        <v>10</v>
+      </c>
+      <c r="E114">
+        <v>306</v>
+      </c>
+      <c r="F114">
+        <v>4</v>
+      </c>
+      <c r="G114">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>46126</v>
+      </c>
+      <c r="B115" t="s">
+        <v>9</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115" t="s">
+        <v>12</v>
+      </c>
+      <c r="E115">
+        <v>192</v>
+      </c>
+      <c r="F115">
+        <v>4</v>
+      </c>
+      <c r="G115">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
+        <v>46127</v>
+      </c>
+      <c r="B116" t="s">
+        <v>9</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116" t="s">
+        <v>6</v>
+      </c>
+      <c r="E116">
+        <v>427</v>
+      </c>
+      <c r="F116">
+        <v>4</v>
+      </c>
+      <c r="G116">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="1">
+        <v>46128</v>
+      </c>
+      <c r="B117" t="s">
+        <v>11</v>
+      </c>
+      <c r="C117" t="s">
+        <v>16</v>
+      </c>
+      <c r="D117" t="s">
+        <v>6</v>
+      </c>
+      <c r="E117">
+        <v>335</v>
+      </c>
+      <c r="F117">
+        <v>4</v>
+      </c>
+      <c r="G117">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="1">
+        <v>46129</v>
+      </c>
+      <c r="B118" t="s">
+        <v>9</v>
+      </c>
+      <c r="C118" t="s">
+        <v>16</v>
+      </c>
+      <c r="D118" t="s">
+        <v>6</v>
+      </c>
+      <c r="E118">
+        <v>79</v>
+      </c>
+      <c r="F118">
+        <v>4</v>
+      </c>
+      <c r="G118">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="1">
+        <v>46130</v>
+      </c>
+      <c r="B119" t="s">
+        <v>9</v>
+      </c>
+      <c r="C119" t="s">
+        <v>16</v>
+      </c>
+      <c r="D119" t="s">
+        <v>6</v>
+      </c>
+      <c r="E119">
+        <v>71</v>
+      </c>
+      <c r="F119">
+        <v>4</v>
+      </c>
+      <c r="G119">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="1">
+        <v>46131</v>
+      </c>
+      <c r="B120" t="s">
+        <v>9</v>
+      </c>
+      <c r="C120" t="s">
+        <v>16</v>
+      </c>
+      <c r="D120" t="s">
+        <v>8</v>
+      </c>
+      <c r="E120">
+        <v>471</v>
+      </c>
+      <c r="F120">
+        <v>4</v>
+      </c>
+      <c r="G120">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A121" s="1">
+        <v>46132</v>
+      </c>
+      <c r="B121" t="s">
+        <v>9</v>
+      </c>
+      <c r="C121" t="s">
+        <v>16</v>
+      </c>
+      <c r="D121" t="s">
+        <v>12</v>
+      </c>
+      <c r="E121">
+        <v>438</v>
+      </c>
+      <c r="F121">
+        <v>4</v>
+      </c>
+      <c r="G121">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="1">
+        <v>46133</v>
+      </c>
+      <c r="B122" t="s">
+        <v>11</v>
+      </c>
+      <c r="C122" t="s">
+        <v>16</v>
+      </c>
+      <c r="D122" t="s">
+        <v>10</v>
+      </c>
+      <c r="E122">
+        <v>187</v>
+      </c>
+      <c r="F122">
+        <v>4</v>
+      </c>
+      <c r="G122">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A123" s="1">
+        <v>46134</v>
+      </c>
+      <c r="B123" t="s">
+        <v>9</v>
+      </c>
+      <c r="C123" t="s">
+        <v>16</v>
+      </c>
+      <c r="D123" t="s">
+        <v>12</v>
+      </c>
+      <c r="E123">
+        <v>497</v>
+      </c>
+      <c r="F123">
+        <v>4</v>
+      </c>
+      <c r="G123">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="1">
+        <v>46135</v>
+      </c>
+      <c r="B124" t="s">
+        <v>5</v>
+      </c>
+      <c r="C124" t="s">
+        <v>16</v>
+      </c>
+      <c r="D124" t="s">
+        <v>10</v>
+      </c>
+      <c r="E124">
+        <v>237</v>
+      </c>
+      <c r="F124">
+        <v>4</v>
+      </c>
+      <c r="G124">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="1">
+        <v>46136</v>
+      </c>
+      <c r="B125" t="s">
+        <v>11</v>
+      </c>
+      <c r="C125" t="s">
+        <v>16</v>
+      </c>
+      <c r="D125" t="s">
+        <v>8</v>
+      </c>
+      <c r="E125">
+        <v>102</v>
+      </c>
+      <c r="F125">
+        <v>4</v>
+      </c>
+      <c r="G125">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A126" s="1">
+        <v>46137</v>
+      </c>
+      <c r="B126" t="s">
+        <v>7</v>
+      </c>
+      <c r="C126" t="s">
+        <v>16</v>
+      </c>
+      <c r="D126" t="s">
+        <v>12</v>
+      </c>
+      <c r="E126">
+        <v>480</v>
+      </c>
+      <c r="F126">
+        <v>4</v>
+      </c>
+      <c r="G126">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A127" s="1">
+        <v>46138</v>
+      </c>
+      <c r="B127" t="s">
+        <v>7</v>
+      </c>
+      <c r="C127" t="s">
+        <v>16</v>
+      </c>
+      <c r="D127" t="s">
+        <v>12</v>
+      </c>
+      <c r="E127">
+        <v>480</v>
+      </c>
+      <c r="F127">
+        <v>4</v>
+      </c>
+      <c r="G127">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="1">
+        <v>46149</v>
+      </c>
+      <c r="B128" t="s">
+        <v>5</v>
+      </c>
+      <c r="C128" t="s">
+        <v>16</v>
+      </c>
+      <c r="D128" t="s">
+        <v>8</v>
+      </c>
+      <c r="E128">
+        <v>101</v>
+      </c>
+      <c r="F128">
+        <v>4</v>
+      </c>
+      <c r="G128">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="1">
+        <v>46150</v>
+      </c>
+      <c r="B129" t="s">
+        <v>5</v>
+      </c>
+      <c r="C129" t="s">
+        <v>16</v>
+      </c>
+      <c r="D129" t="s">
+        <v>10</v>
+      </c>
+      <c r="E129">
+        <v>356</v>
+      </c>
+      <c r="F129">
+        <v>4</v>
+      </c>
+      <c r="G129">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="1">
+        <v>46151</v>
+      </c>
+      <c r="B130" t="s">
+        <v>9</v>
+      </c>
+      <c r="C130" t="s">
+        <v>16</v>
+      </c>
+      <c r="D130" t="s">
+        <v>8</v>
+      </c>
+      <c r="E130">
+        <v>208</v>
+      </c>
+      <c r="F130">
+        <v>4</v>
+      </c>
+      <c r="G130">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="1">
+        <v>46183</v>
+      </c>
+      <c r="B131" t="s">
+        <v>7</v>
+      </c>
+      <c r="C131" t="s">
+        <v>16</v>
+      </c>
+      <c r="D131" t="s">
+        <v>6</v>
+      </c>
+      <c r="E131">
+        <v>76</v>
+      </c>
+      <c r="F131">
+        <v>4</v>
+      </c>
+      <c r="G131">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="1">
+        <v>46184</v>
+      </c>
+      <c r="B132" t="s">
+        <v>7</v>
+      </c>
+      <c r="C132" t="s">
+        <v>16</v>
+      </c>
+      <c r="D132" t="s">
+        <v>6</v>
+      </c>
+      <c r="E132">
+        <v>261</v>
+      </c>
+      <c r="F132">
+        <v>4</v>
+      </c>
+      <c r="G132">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="1">
+        <v>46185</v>
+      </c>
+      <c r="B133" t="s">
+        <v>7</v>
+      </c>
+      <c r="C133" t="s">
+        <v>16</v>
+      </c>
+      <c r="D133" t="s">
+        <v>6</v>
+      </c>
+      <c r="E133">
+        <v>205</v>
+      </c>
+      <c r="F133">
+        <v>4</v>
+      </c>
+      <c r="G133">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="1">
+        <v>46186</v>
+      </c>
+      <c r="B134" t="s">
+        <v>11</v>
+      </c>
+      <c r="C134" t="s">
+        <v>16</v>
+      </c>
+      <c r="D134" t="s">
+        <v>10</v>
+      </c>
+      <c r="E134">
+        <v>306</v>
+      </c>
+      <c r="F134">
+        <v>4</v>
+      </c>
+      <c r="G134">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A135" s="1">
+        <v>46217</v>
+      </c>
+      <c r="B135" t="s">
+        <v>9</v>
+      </c>
+      <c r="C135" t="s">
+        <v>16</v>
+      </c>
+      <c r="D135" t="s">
+        <v>12</v>
+      </c>
+      <c r="E135">
+        <v>192</v>
+      </c>
+      <c r="F135">
+        <v>4</v>
+      </c>
+      <c r="G135">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B136" t="s">
+        <v>9</v>
+      </c>
+      <c r="C136" t="s">
+        <v>16</v>
+      </c>
+      <c r="D136" t="s">
+        <v>6</v>
+      </c>
+      <c r="E136">
+        <v>427</v>
+      </c>
+      <c r="F136">
+        <v>4</v>
+      </c>
+      <c r="G136">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="1">
+        <v>46219</v>
+      </c>
+      <c r="B137" t="s">
+        <v>11</v>
+      </c>
+      <c r="C137" t="s">
+        <v>16</v>
+      </c>
+      <c r="D137" t="s">
+        <v>6</v>
+      </c>
+      <c r="E137">
+        <v>335</v>
+      </c>
+      <c r="F137">
+        <v>4</v>
+      </c>
+      <c r="G137">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="1">
+        <v>46251</v>
+      </c>
+      <c r="B138" t="s">
+        <v>9</v>
+      </c>
+      <c r="C138" t="s">
+        <v>16</v>
+      </c>
+      <c r="D138" t="s">
+        <v>6</v>
+      </c>
+      <c r="E138">
+        <v>79</v>
+      </c>
+      <c r="F138">
+        <v>4</v>
+      </c>
+      <c r="G138">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="1">
+        <v>46252</v>
+      </c>
+      <c r="B139" t="s">
+        <v>9</v>
+      </c>
+      <c r="C139" t="s">
+        <v>16</v>
+      </c>
+      <c r="D139" t="s">
+        <v>6</v>
+      </c>
+      <c r="E139">
+        <v>71</v>
+      </c>
+      <c r="F139">
+        <v>4</v>
+      </c>
+      <c r="G139">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B140" t="s">
+        <v>9</v>
+      </c>
+      <c r="C140" t="s">
+        <v>16</v>
+      </c>
+      <c r="D140" t="s">
+        <v>8</v>
+      </c>
+      <c r="E140">
+        <v>471</v>
+      </c>
+      <c r="F140">
+        <v>4</v>
+      </c>
+      <c r="G140">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A141" s="1">
+        <v>46254</v>
+      </c>
+      <c r="B141" t="s">
+        <v>9</v>
+      </c>
+      <c r="C141" t="s">
+        <v>16</v>
+      </c>
+      <c r="D141" t="s">
+        <v>12</v>
+      </c>
+      <c r="E141">
+        <v>438</v>
+      </c>
+      <c r="F141">
+        <v>4</v>
+      </c>
+      <c r="G141">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="1">
+        <v>46286</v>
+      </c>
+      <c r="B142" t="s">
+        <v>11</v>
+      </c>
+      <c r="C142" t="s">
+        <v>16</v>
+      </c>
+      <c r="D142" t="s">
+        <v>10</v>
+      </c>
+      <c r="E142">
+        <v>187</v>
+      </c>
+      <c r="F142">
+        <v>4</v>
+      </c>
+      <c r="G142">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A143" s="1">
+        <v>46287</v>
+      </c>
+      <c r="B143" t="s">
+        <v>9</v>
+      </c>
+      <c r="C143" t="s">
+        <v>16</v>
+      </c>
+      <c r="D143" t="s">
+        <v>12</v>
+      </c>
+      <c r="E143">
+        <v>497</v>
+      </c>
+      <c r="F143">
+        <v>4</v>
+      </c>
+      <c r="G143">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="1">
+        <v>46288</v>
+      </c>
+      <c r="B144" t="s">
+        <v>5</v>
+      </c>
+      <c r="C144" t="s">
+        <v>16</v>
+      </c>
+      <c r="D144" t="s">
+        <v>10</v>
+      </c>
+      <c r="E144">
+        <v>237</v>
+      </c>
+      <c r="F144">
+        <v>4</v>
+      </c>
+      <c r="G144">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="1">
+        <v>46289</v>
+      </c>
+      <c r="B145" t="s">
+        <v>11</v>
+      </c>
+      <c r="C145" t="s">
+        <v>16</v>
+      </c>
+      <c r="D145" t="s">
+        <v>8</v>
+      </c>
+      <c r="E145">
+        <v>102</v>
+      </c>
+      <c r="F145">
+        <v>4</v>
+      </c>
+      <c r="G145">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A146" s="1">
+        <v>46320</v>
+      </c>
+      <c r="B146" t="s">
+        <v>7</v>
+      </c>
+      <c r="C146" t="s">
+        <v>16</v>
+      </c>
+      <c r="D146" t="s">
+        <v>12</v>
+      </c>
+      <c r="E146">
+        <v>1000</v>
+      </c>
+      <c r="F146">
+        <v>4</v>
+      </c>
+      <c r="G146">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A147" s="1">
+        <v>46321</v>
+      </c>
+      <c r="B147" t="s">
+        <v>7</v>
+      </c>
+      <c r="C147" t="s">
+        <v>16</v>
+      </c>
+      <c r="D147" t="s">
+        <v>12</v>
+      </c>
+      <c r="E147">
+        <v>480</v>
+      </c>
+      <c r="F147">
+        <v>4</v>
+      </c>
+      <c r="G147">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A148" s="1">
+        <v>45767</v>
+      </c>
+      <c r="B148" t="s">
+        <v>9</v>
+      </c>
+      <c r="C148" t="s">
+        <v>16</v>
+      </c>
+      <c r="D148" t="s">
+        <v>12</v>
+      </c>
+      <c r="E148">
+        <v>438</v>
+      </c>
+      <c r="F148">
+        <v>4</v>
+      </c>
+      <c r="G148">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="1">
+        <v>45768</v>
+      </c>
+      <c r="B149" t="s">
+        <v>11</v>
+      </c>
+      <c r="C149" t="s">
+        <v>16</v>
+      </c>
+      <c r="D149" t="s">
+        <v>10</v>
+      </c>
+      <c r="E149">
+        <v>187</v>
+      </c>
+      <c r="F149">
+        <v>4</v>
+      </c>
+      <c r="G149">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A150" s="1">
+        <v>45769</v>
+      </c>
+      <c r="B150" t="s">
+        <v>9</v>
+      </c>
+      <c r="C150" t="s">
+        <v>16</v>
+      </c>
+      <c r="D150" t="s">
+        <v>12</v>
+      </c>
+      <c r="E150">
+        <v>497</v>
+      </c>
+      <c r="F150">
+        <v>4</v>
+      </c>
+      <c r="G150">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="1">
+        <v>45770</v>
+      </c>
+      <c r="B151" t="s">
+        <v>5</v>
+      </c>
+      <c r="C151" t="s">
+        <v>16</v>
+      </c>
+      <c r="D151" t="s">
+        <v>10</v>
+      </c>
+      <c r="E151">
+        <v>237</v>
+      </c>
+      <c r="F151">
+        <v>4</v>
+      </c>
+      <c r="G151">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="1">
+        <v>45771</v>
+      </c>
+      <c r="B152" t="s">
+        <v>11</v>
+      </c>
+      <c r="C152" t="s">
+        <v>16</v>
+      </c>
+      <c r="D152" t="s">
+        <v>8</v>
+      </c>
+      <c r="E152">
+        <v>102</v>
+      </c>
+      <c r="F152">
+        <v>4</v>
+      </c>
+      <c r="G152">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A153" s="1">
+        <v>45772</v>
+      </c>
+      <c r="B153" t="s">
+        <v>7</v>
+      </c>
+      <c r="C153" t="s">
+        <v>16</v>
+      </c>
+      <c r="D153" t="s">
+        <v>12</v>
+      </c>
+      <c r="E153">
+        <v>480</v>
+      </c>
+      <c r="F153">
+        <v>4</v>
+      </c>
+      <c r="G153">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" s="1">
+        <v>45773</v>
+      </c>
+      <c r="B154" t="s">
+        <v>7</v>
+      </c>
+      <c r="C154" t="s">
+        <v>16</v>
+      </c>
+      <c r="D154" t="s">
+        <v>12</v>
+      </c>
+      <c r="E154">
+        <v>480</v>
+      </c>
+      <c r="F154">
+        <v>4</v>
+      </c>
+      <c r="G154">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="1">
+        <v>45784</v>
+      </c>
+      <c r="B155" t="s">
+        <v>5</v>
+      </c>
+      <c r="C155" t="s">
+        <v>16</v>
+      </c>
+      <c r="D155" t="s">
+        <v>8</v>
+      </c>
+      <c r="E155">
+        <v>101</v>
+      </c>
+      <c r="F155">
+        <v>4</v>
+      </c>
+      <c r="G155">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="1">
+        <v>45785</v>
+      </c>
+      <c r="B156" t="s">
+        <v>5</v>
+      </c>
+      <c r="C156" t="s">
+        <v>16</v>
+      </c>
+      <c r="D156" t="s">
+        <v>10</v>
+      </c>
+      <c r="E156">
+        <v>356</v>
+      </c>
+      <c r="F156">
+        <v>4</v>
+      </c>
+      <c r="G156">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="1">
+        <v>45786</v>
+      </c>
+      <c r="B157" t="s">
+        <v>9</v>
+      </c>
+      <c r="C157" t="s">
+        <v>16</v>
+      </c>
+      <c r="D157" t="s">
+        <v>8</v>
+      </c>
+      <c r="E157">
+        <v>208</v>
+      </c>
+      <c r="F157">
+        <v>4</v>
+      </c>
+      <c r="G157">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="1">
+        <v>45818</v>
+      </c>
+      <c r="B158" t="s">
+        <v>7</v>
+      </c>
+      <c r="C158" t="s">
+        <v>16</v>
+      </c>
+      <c r="D158" t="s">
+        <v>6</v>
+      </c>
+      <c r="E158">
+        <v>76</v>
+      </c>
+      <c r="F158">
+        <v>4</v>
+      </c>
+      <c r="G158">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B159" t="s">
+        <v>7</v>
+      </c>
+      <c r="C159" t="s">
+        <v>16</v>
+      </c>
+      <c r="D159" t="s">
+        <v>6</v>
+      </c>
+      <c r="E159">
+        <v>261</v>
+      </c>
+      <c r="F159">
+        <v>4</v>
+      </c>
+      <c r="G159">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="1">
+        <v>45820</v>
+      </c>
+      <c r="B160" t="s">
+        <v>7</v>
+      </c>
+      <c r="C160" t="s">
+        <v>16</v>
+      </c>
+      <c r="D160" t="s">
+        <v>6</v>
+      </c>
+      <c r="E160">
+        <v>205</v>
+      </c>
+      <c r="F160">
+        <v>4</v>
+      </c>
+      <c r="G160">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="1">
+        <v>45821</v>
+      </c>
+      <c r="B161" t="s">
+        <v>11</v>
+      </c>
+      <c r="C161" t="s">
+        <v>16</v>
+      </c>
+      <c r="D161" t="s">
+        <v>10</v>
+      </c>
+      <c r="E161">
+        <v>306</v>
+      </c>
+      <c r="F161">
+        <v>4</v>
+      </c>
+      <c r="G161">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" s="1">
+        <v>45852</v>
+      </c>
+      <c r="B162" t="s">
+        <v>9</v>
+      </c>
+      <c r="C162" t="s">
+        <v>16</v>
+      </c>
+      <c r="D162" t="s">
+        <v>12</v>
+      </c>
+      <c r="E162">
+        <v>192</v>
+      </c>
+      <c r="F162">
+        <v>4</v>
+      </c>
+      <c r="G162">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="1">
+        <v>45853</v>
+      </c>
+      <c r="B163" t="s">
+        <v>9</v>
+      </c>
+      <c r="C163" t="s">
+        <v>16</v>
+      </c>
+      <c r="D163" t="s">
+        <v>6</v>
+      </c>
+      <c r="E163">
+        <v>427</v>
+      </c>
+      <c r="F163">
+        <v>4</v>
+      </c>
+      <c r="G163">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="1">
+        <v>45854</v>
+      </c>
+      <c r="B164" t="s">
+        <v>11</v>
+      </c>
+      <c r="C164" t="s">
+        <v>16</v>
+      </c>
+      <c r="D164" t="s">
+        <v>6</v>
+      </c>
+      <c r="E164">
+        <v>335</v>
+      </c>
+      <c r="F164">
+        <v>4</v>
+      </c>
+      <c r="G164">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="1">
+        <v>45855</v>
+      </c>
+      <c r="B165" t="s">
+        <v>9</v>
+      </c>
+      <c r="C165" t="s">
+        <v>16</v>
+      </c>
+      <c r="D165" t="s">
+        <v>6</v>
+      </c>
+      <c r="E165">
+        <v>79</v>
+      </c>
+      <c r="F165">
+        <v>4</v>
+      </c>
+      <c r="G165">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="1">
+        <v>45887</v>
+      </c>
+      <c r="B166" t="s">
+        <v>9</v>
+      </c>
+      <c r="C166" t="s">
+        <v>16</v>
+      </c>
+      <c r="D166" t="s">
+        <v>6</v>
+      </c>
+      <c r="E166">
+        <v>71</v>
+      </c>
+      <c r="F166">
+        <v>4</v>
+      </c>
+      <c r="G166">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="1">
+        <v>45888</v>
+      </c>
+      <c r="B167" t="s">
+        <v>9</v>
+      </c>
+      <c r="C167" t="s">
+        <v>16</v>
+      </c>
+      <c r="D167" t="s">
+        <v>8</v>
+      </c>
+      <c r="E167">
+        <v>471</v>
+      </c>
+      <c r="F167">
+        <v>4</v>
+      </c>
+      <c r="G167">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A168" s="1">
+        <v>45889</v>
+      </c>
+      <c r="B168" t="s">
+        <v>9</v>
+      </c>
+      <c r="C168" t="s">
+        <v>16</v>
+      </c>
+      <c r="D168" t="s">
+        <v>12</v>
+      </c>
+      <c r="E168">
+        <v>438</v>
+      </c>
+      <c r="F168">
+        <v>4</v>
+      </c>
+      <c r="G168">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A169" s="1">
+        <v>45921</v>
+      </c>
+      <c r="B169" t="s">
+        <v>11</v>
+      </c>
+      <c r="C169" t="s">
+        <v>16</v>
+      </c>
+      <c r="D169" t="s">
+        <v>10</v>
+      </c>
+      <c r="E169">
+        <v>187</v>
+      </c>
+      <c r="F169">
+        <v>4</v>
+      </c>
+      <c r="G169">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A170" s="1">
+        <v>45922</v>
+      </c>
+      <c r="B170" t="s">
+        <v>9</v>
+      </c>
+      <c r="C170" t="s">
+        <v>16</v>
+      </c>
+      <c r="D170" t="s">
+        <v>12</v>
+      </c>
+      <c r="E170">
+        <v>497</v>
+      </c>
+      <c r="F170">
+        <v>4</v>
+      </c>
+      <c r="G170">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="1">
+        <v>45923</v>
+      </c>
+      <c r="B171" t="s">
+        <v>5</v>
+      </c>
+      <c r="C171" t="s">
+        <v>16</v>
+      </c>
+      <c r="D171" t="s">
+        <v>10</v>
+      </c>
+      <c r="E171">
+        <v>237</v>
+      </c>
+      <c r="F171">
+        <v>4</v>
+      </c>
+      <c r="G171">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="1">
+        <v>45924</v>
+      </c>
+      <c r="B172" t="s">
+        <v>11</v>
+      </c>
+      <c r="C172" t="s">
+        <v>16</v>
+      </c>
+      <c r="D172" t="s">
+        <v>8</v>
+      </c>
+      <c r="E172">
+        <v>102</v>
+      </c>
+      <c r="F172">
+        <v>4</v>
+      </c>
+      <c r="G172">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A173" s="1">
+        <v>45955</v>
+      </c>
+      <c r="B173" t="s">
+        <v>7</v>
+      </c>
+      <c r="C173" t="s">
+        <v>16</v>
+      </c>
+      <c r="D173" t="s">
+        <v>12</v>
+      </c>
+      <c r="E173">
+        <v>1000</v>
+      </c>
+      <c r="F173">
+        <v>4</v>
+      </c>
+      <c r="G173">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A174" s="1">
+        <v>45956</v>
+      </c>
+      <c r="B174" t="s">
+        <v>7</v>
+      </c>
+      <c r="C174" t="s">
+        <v>16</v>
+      </c>
+      <c r="D174" t="s">
+        <v>12</v>
+      </c>
+      <c r="E174">
+        <v>480</v>
+      </c>
+      <c r="F174">
+        <v>4</v>
+      </c>
+      <c r="G174">
+        <v>0.02</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E101" xr:uid="{8619DC5A-B133-4640-889F-547BAA264472}">
-    <filterColumn colId="2">
+  <autoFilter ref="A1:G174" xr:uid="{8619DC5A-B133-4640-889F-547BAA264472}">
+    <filterColumn colId="3">
       <filters>
-        <filter val="PR"/>
+        <filter val="Ana"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB15C8C2-938D-49B1-B8B7-551F3275220F}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>17000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>